<commit_message>
SP500 als fester Index im Notebook hinzugefügt und Testdaten angepasst
</commit_message>
<xml_diff>
--- a/notebooks/credit/test_data/Datenmodell_Krediportfoliomodell_test.xlsx
+++ b/notebooks/credit/test_data/Datenmodell_Krediportfoliomodell_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anwender\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Noah Köstner\repos_vscode\RiVaPy\notebooks\credit\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E4BCEA-1EAC-45BC-A4D9-0C136FF8D004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F37CDA-7226-4C27-9CC5-B7E73D2AAA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A210388-5C51-485A-97F5-F242A4A15662}"/>
+    <workbookView xWindow="1548" yWindow="1548" windowWidth="17280" windowHeight="8880" xr2:uid="{1A210388-5C51-485A-97F5-F242A4A15662}"/>
   </bookViews>
   <sheets>
     <sheet name="Positions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>InstrumentID</t>
   </si>
@@ -102,7 +102,10 @@
     <t>Industrials</t>
   </si>
   <si>
-    <t>Issuer_4</t>
+    <t>US</t>
+  </si>
+  <si>
+    <t>GM</t>
   </si>
 </sst>
 </file>
@@ -164,8 +167,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -514,15 +517,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{554CDDF5-67C6-4311-98F8-AD12F58EF367}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.86328125" customWidth="1"/>
-    <col min="2" max="2" width="18.26953125" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" customWidth="1"/>
-    <col min="6" max="6" width="15.26953125" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -542,7 +545,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -563,7 +566,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -584,7 +587,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -605,7 +608,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -626,7 +629,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -647,7 +650,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -668,7 +671,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -689,7 +692,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -701,7 +704,7 @@
         <v>300000</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -710,7 +713,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -722,7 +725,7 @@
         <v>300000</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -731,7 +734,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -763,13 +766,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29C9E912-4BAC-42CB-975A-18BE9AD025E1}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.7265625" customWidth="1"/>
-    <col min="4" max="4" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -786,7 +789,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -803,7 +806,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -820,7 +823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -837,18 +840,18 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
@@ -858,7 +861,7 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="B2:B5" calculatedColumn="1"/>
+    <ignoredError sqref="B2:B4" calculatedColumn="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
@@ -869,9 +872,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A0A61E-6BDF-4593-8C1C-042B01910D72}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>10</v>
       </c>

</xml_diff>